<commit_message>
Correcciones JPGE a JPEG. Se agregó un convertidor de coordenadas UTM a latitud y longitud.
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/AvistamientoFauna/Formato de Descarga de Datos.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/AvistamientoFauna/Formato de Descarga de Datos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Segunda Etapa\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\AvistamientoFauna\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Segunda Etapa\AvistamientoFauna\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\AvistamientoFauna\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D7277FC-A627-45B4-85DF-B2F11BCB2636}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9CE161-38B4-4E66-8D5F-8EA8CA3B6315}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6D4A8E67-509A-4493-8736-F3C59B5C1B98}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Item</t>
   </si>
@@ -72,6 +72,15 @@
   </si>
   <si>
     <t>Código</t>
+  </si>
+  <si>
+    <t>Latitud (Lugar Referencia)</t>
+  </si>
+  <si>
+    <t>Longitud (Lugar Referencia)</t>
+  </si>
+  <si>
+    <t>Link Google Maps (Lugar Referencia)</t>
   </si>
 </sst>
 </file>
@@ -159,7 +168,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -455,8 +464,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{212B9101-7E31-46E2-B23C-DD724D576579}">
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
@@ -471,9 +480,10 @@
     <col min="11" max="11" width="26.7109375" customWidth="1"/>
     <col min="12" max="12" width="25" customWidth="1"/>
     <col min="13" max="13" width="27.7109375" customWidth="1"/>
+    <col min="14" max="16" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,6 +522,15 @@
       </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>